<commit_message>
docs(trazabilidad): reconcile RF-013/RF-014 across sprint and traceability docs
RF-013 (interoperabilidad institucional) y RF-014 (wearables como validación
clínica) se habían agregado al SRS/SAD pero no estaban reflejados en la
Matriz de Trazabilidad, el plan de Sprint 13 ni el Informe de
Trazabilidad SRS-SAD-Implementación. Se agregan sus bloques/secciones en
los tres artefactos, incluyendo la evidencia de código real y la nota
honesta de que ninguno de los dos cuenta con diagrama UML dedicado.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Documentation/trazabilidad/Matriz_Trazabilidad_RespiCare.xlsx
+++ b/Documentation/trazabilidad/Matriz_Trazabilidad_RespiCare.xlsx
@@ -537,7 +537,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F76"/>
+  <dimension ref="A1:F88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -566,7 +566,7 @@
     <row r="3" ht="120" customHeight="1">
       <c r="A3" s="11" t="inlineStr">
         <is>
-          <t>Orden y justificación de las filas (por requerimiento): Diagrama de Paquetes -&gt; Diagrama de Casos de Uso -&gt; Diagrama de Clases -&gt; Diagrama de Secuencia -&gt; Diagrama de Actividades -&gt; Diagrama de Entidad-Relación (lógico). El orden reproduce el recorrido metodológico de afuera hacia adentro y de lo estático a lo persistente: (1) Paquetes delimita el módulo del sistema donde vive el requerimiento (organización); (2) Casos de Uso define QUÉ hace el sistema para el actor dentro de ese módulo (función); (3) Clases identifica, a partir del caso de uso, los objetos del dominio y sus relaciones estáticas (estructura); (4) Secuencia detalla CÓMO interactúan esas clases en el tiempo para resolver el escenario (comportamiento interno); (5) Actividades complementa la secuencia con el flujo de proceso/negocio y sus decisiones o excepciones (comportamiento de proceso); (6) Entidad-Relación (lógico) cierra la cadena derivando el modelo de datos persistente (colecciones MongoDB) a partir de las clases de dominio ya identificadas, conectando el análisis y el diseño con la capa de persistencia real documentada en el SAD (§10.1). Aplicar este mismo orden en las 12 filas de requerimientos permite comparar, RF a RF, en qué eslabón de la cadena existe o no evidencia verificable en el código.</t>
+          <t>Orden y justificación de las filas (por requerimiento): Diagrama de Paquetes -&gt; Diagrama de Casos de Uso -&gt; Diagrama de Clases -&gt; Diagrama de Secuencia -&gt; Diagrama de Actividades -&gt; Diagrama de Entidad-Relación (lógico). El orden reproduce el recorrido metodológico de afuera hacia adentro y de lo estático a lo persistente: (1) Paquetes delimita el módulo del sistema donde vive el requerimiento (organización); (2) Casos de Uso define QUÉ hace el sistema para el actor dentro de ese módulo (función); (3) Clases identifica, a partir del caso de uso, los objetos del dominio y sus relaciones estáticas (estructura); (4) Secuencia detalla CÓMO interactúan esas clases en el tiempo para resolver el escenario (comportamiento interno); (5) Actividades complementa la secuencia con el flujo de proceso/negocio y sus decisiones o excepciones (comportamiento de proceso); (6) Entidad-Relación (lógico) cierra la cadena derivando el modelo de datos persistente (colecciones MongoDB) a partir de las clases de dominio ya identificadas, conectando el análisis y el diseño con la capa de persistencia real documentada en el SAD (§10.1). Aplicar este mismo orden en las 14 filas de requerimientos permite comparar, RF a RF, en qué eslabón de la cadena existe o no evidencia verificable en el código.</t>
         </is>
       </c>
     </row>
@@ -2687,6 +2687,334 @@
         </is>
       </c>
       <c r="F76" s="10" t="n"/>
+    </row>
+    <row r="77" ht="80" customHeight="1">
+      <c r="A77" s="4" t="inlineStr">
+        <is>
+          <t>RF-013: "Interoperabilidad institucional (MINSA/DIRESA/SINADEF)"
+(CU-015: Consultar datos epidemiológicos institucionales)</t>
+        </is>
+      </c>
+      <c r="B77" s="5" t="inlineStr">
+        <is>
+          <t>N/A — no se elaboró un Diagrama de Paquetes dedicado para este requerimiento; el análisis se documenta como narrativa de caso de uso CU-015 (FD03, tabla de casos de uso — sin figura numerada, agregada en Sprint 13).</t>
+        </is>
+      </c>
+      <c r="C77" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D77" s="5" t="inlineStr">
+        <is>
+          <t>N/A — no se elaboró un Diagrama de Paquetes dedicado; el diseño se documenta como narrativa de caso de uso CU-006 (FD04, antes de §6 Vista Lógica — sin figura numerada, agregada en Sprint 13).</t>
+        </is>
+      </c>
+      <c r="E77" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F77" s="7" t="inlineStr">
+        <is>
+          <t>Objetos de programación creados (Sprint 13):
+Backend (backend/src) — API institucional autenticada por API Key (no JWT):
+• routes/institutionalRoutes.ts — GET /epidemiological-export, POST /health-centers/sync, POST /alerts, montadas en /api/v1/institutional (index.ts:297)
+• middleware/institutionalAuth.ts — authenticateInstitutional() valida el header x-api-key contra InstitutionalApiClient.verifyKey(); requireInstitutionalScope(scope) verifica el alcance autorizado; institutionalRateLimiter limita solicitudes por API Key
+• controllers/institutionalController.ts — getEpidemiologicalExport(), syncHealthCenters(), ingestAlert()
+• services/institutionalIntegrationService.ts — getEpidemiologicalExport() reutiliza epidemiologicalService.getDistrictTrends()/predictOutbreaks(); syncHealthCenters() hace upsert por nombre+distrito; ingestExternalAlert() crea un Alert (categoría health_authority) por cada médico/admin activo
+• models/InstitutionalApiClient.ts — colección institutionalapiclients: keyHash, scopes[] (epidemiological:read, health-centers:write, alerts:write), verifyKey()
+• models/InstitutionalAuditLog.ts — colección institutionalauditlogs: bitácora independiente de todo el tráfico institucional (clientId, método, ruta, statusCode)
+• openapi/institutional-api.yaml — contrato OpenAPI del API institucional
+• scripts/generateInstitutionalApiKey.ts — script de aprovisionamiento de API Keys institucionales</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="80" customHeight="1">
+      <c r="A78" s="9" t="n"/>
+      <c r="B78" s="5" t="inlineStr">
+        <is>
+          <t>CU-015: "Consultar datos epidemiológicos institucionales" — Actor: Sistema institucional externo (MINSA/DIRESA/SINADEF) (FD03).</t>
+        </is>
+      </c>
+      <c r="C78" s="6" t="inlineStr">
+        <is>
+          <t>→ Base para</t>
+        </is>
+      </c>
+      <c r="D78" s="5" t="inlineStr">
+        <is>
+          <t>CU-006: "Consulta institucional de datos epidemiológicos (MINSA/DIRESA/SINADEF)" (FD04).</t>
+        </is>
+      </c>
+      <c r="E78" s="6" t="inlineStr">
+        <is>
+          <t>→ Base para</t>
+        </is>
+      </c>
+      <c r="F78" s="9" t="n"/>
+    </row>
+    <row r="79" ht="80" customHeight="1">
+      <c r="A79" s="9" t="n"/>
+      <c r="B79" s="5" t="inlineStr">
+        <is>
+          <t>N/A — no se elaboró un Diagrama de Clases dedicado para este requerimiento; el análisis se documenta como narrativa de caso de uso CU-015 (FD03, tabla de casos de uso — sin figura numerada, agregada en Sprint 13).</t>
+        </is>
+      </c>
+      <c r="C79" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D79" s="5" t="inlineStr">
+        <is>
+          <t>N/A — no se elaboró un Diagrama de Clases dedicado; el diseño se documenta como narrativa de caso de uso CU-006 (FD04, antes de §6 Vista Lógica — sin figura numerada, agregada en Sprint 13).</t>
+        </is>
+      </c>
+      <c r="E79" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F79" s="9" t="n"/>
+    </row>
+    <row r="80" ht="80" customHeight="1">
+      <c r="A80" s="9" t="n"/>
+      <c r="B80" s="5" t="inlineStr">
+        <is>
+          <t>N/A — no se elaboró un Diagrama de Secuencia dedicado para este requerimiento; el análisis se documenta como narrativa de caso de uso CU-015 (FD03, tabla de casos de uso — sin figura numerada, agregada en Sprint 13).</t>
+        </is>
+      </c>
+      <c r="C80" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D80" s="5" t="inlineStr">
+        <is>
+          <t>N/A — no se elaboró un Diagrama de Secuencia dedicado; el diseño se documenta como narrativa de caso de uso CU-006 (FD04, antes de §6 Vista Lógica — sin figura numerada, agregada en Sprint 13).</t>
+        </is>
+      </c>
+      <c r="E80" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F80" s="9" t="n"/>
+    </row>
+    <row r="81" ht="80" customHeight="1">
+      <c r="A81" s="9" t="n"/>
+      <c r="B81" s="5" t="inlineStr">
+        <is>
+          <t>N/A — no se elaboró un Diagrama de Actividades dedicado para este requerimiento; el análisis se documenta como narrativa de caso de uso CU-015 (FD03, tabla de casos de uso — sin figura numerada, agregada en Sprint 13).</t>
+        </is>
+      </c>
+      <c r="C81" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D81" s="5" t="inlineStr">
+        <is>
+          <t>N/A — no se elaboró un Diagrama de Actividades dedicado; el diseño se documenta como narrativa de caso de uso CU-006 (FD04, antes de §6 Vista Lógica — sin figura numerada, agregada en Sprint 13).</t>
+        </is>
+      </c>
+      <c r="E81" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F81" s="9" t="n"/>
+    </row>
+    <row r="82" ht="155" customHeight="1">
+      <c r="A82" s="10" t="n"/>
+      <c r="B82" s="5" t="inlineStr">
+        <is>
+          <t>N/A — el SRS (FD03) documenta el requerimiento a nivel de caso de uso; el modelo de datos persistente se define en la fase de diseño (FD04).</t>
+        </is>
+      </c>
+      <c r="C82" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D82" s="5" t="inlineStr">
+        <is>
+          <t>Diagrama de Entidad-Relación (lógico) — Base de Datos MongoDB.
+Entidades nuevas "INSTITUTIONAL_API_CLIENTS" (colección institutionalapiclients) e "INSTITUTIONAL_AUDIT_LOGS" (colección institutionalauditlogs), no representadas en el Diagrama de Entidad-Relación documentado en DIAGRAMAS_MERMAID.md §4 — brecha de documentación detectada al construir esta fila, análoga a la registrada para ALERTS/AUTOMATIC_REPORTS antes de la ampliación de dicho diagrama. Los datos epidemiológicos exportados no tienen colección propia: se derivan en tiempo real de SYMPTOM_REPORTS/AI_ANALYSES vía epidemiologicalService.</t>
+        </is>
+      </c>
+      <c r="E82" s="6" t="inlineStr">
+        <is>
+          <t>→ Base para</t>
+        </is>
+      </c>
+      <c r="F82" s="10" t="n"/>
+    </row>
+    <row r="83" ht="80" customHeight="1">
+      <c r="A83" s="4" t="inlineStr">
+        <is>
+          <t>RF-014: "Wearables como capa de validación clínica"
+(CU-016: Validar predicción de IA con signos vitales del wearable)</t>
+        </is>
+      </c>
+      <c r="B83" s="5" t="inlineStr">
+        <is>
+          <t>N/A — no se elaboró un Diagrama de Paquetes dedicado para este requerimiento; el análisis se documenta como narrativa de caso de uso CU-016 (FD03, tabla de casos de uso — sin figura numerada, agregada en Sprint 13).</t>
+        </is>
+      </c>
+      <c r="C83" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D83" s="5" t="inlineStr">
+        <is>
+          <t>N/A — no se elaboró un Diagrama de Paquetes dedicado; el diseño se documenta como narrativa de caso de uso CU-007 (FD04, antes de §6 Vista Lógica — sin figura numerada, agregada en Sprint 13).</t>
+        </is>
+      </c>
+      <c r="E83" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F83" s="7" t="inlineStr">
+        <is>
+          <t>Objetos de programación creados (Sprint 13):
+Servicio de IA (ai-services, Python):
+• services/medical_validation_rules.py — MedicalValidationRules.validate_vitals(vitals): evalúa SpO2, frecuencia respiratoria y frecuencia cardíaca contra umbrales clínicos; ajusta confidence_adjustment y puede activar urgency_escalation, sin reemplazar el modelo de ML
+• api/routes/symptom_ml_analyzer.py — _apply_medical_validation(response, symptoms_str, patient_age, vitals=vitals_dict) invoca validate_vitals() en las tres rutas de predicción de /v1/ml-analyze (ensemble, fallback SHAP, fallback por patrones), con degradación automática al comportamiento actual si no hay datos de wearables
+Backend (backend/src):
+• models/WearableData.ts — colección wearabledata: heartRate, oxygenSaturation, respiratoryRate, steps, distance, sleepHours, source (apple_health/google_fit/manual/android_sensor)
+• controllers/wearableController.ts — syncWearableData() persiste cada lectura y emite vitalsEmitter.emit('vitals', ...) para el panel del médico en tiempo real
+• routes/wearableRoutes.ts — POST /sync, GET /data/:patientId?, GET /metrics/:patientId?
+Frontend (web/src):
+• pages/PatientMonitoringPage.js — gráfico de tendencia de SpO2 de 7 días a partir de los datos de wearables sincronizados
+Mobile (mobile/medical-app):
+• lib/api/services/wearableService.ts, lib/services/wearableWebSocket.ts, components/tabs/wearables.tsx — captura BLE/Health Connect/HealthKit y sincronización</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="80" customHeight="1">
+      <c r="A84" s="9" t="n"/>
+      <c r="B84" s="5" t="inlineStr">
+        <is>
+          <t>CU-016: "Validar predicción de IA con signos vitales del wearable" — Actor: Paciente / Sistema de IA (FD03).</t>
+        </is>
+      </c>
+      <c r="C84" s="6" t="inlineStr">
+        <is>
+          <t>→ Base para</t>
+        </is>
+      </c>
+      <c r="D84" s="5" t="inlineStr">
+        <is>
+          <t>CU-007: "Validación de predicción con datos de wearables" (FD04).</t>
+        </is>
+      </c>
+      <c r="E84" s="6" t="inlineStr">
+        <is>
+          <t>→ Base para</t>
+        </is>
+      </c>
+      <c r="F84" s="9" t="n"/>
+    </row>
+    <row r="85" ht="80" customHeight="1">
+      <c r="A85" s="9" t="n"/>
+      <c r="B85" s="5" t="inlineStr">
+        <is>
+          <t>N/A — no se elaboró un Diagrama de Clases dedicado para este requerimiento; el análisis se documenta como narrativa de caso de uso CU-016 (FD03, tabla de casos de uso — sin figura numerada, agregada en Sprint 13).</t>
+        </is>
+      </c>
+      <c r="C85" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D85" s="5" t="inlineStr">
+        <is>
+          <t>N/A — no se elaboró un Diagrama de Clases dedicado; el diseño se documenta como narrativa de caso de uso CU-007 (FD04, antes de §6 Vista Lógica — sin figura numerada, agregada en Sprint 13).</t>
+        </is>
+      </c>
+      <c r="E85" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F85" s="9" t="n"/>
+    </row>
+    <row r="86" ht="80" customHeight="1">
+      <c r="A86" s="9" t="n"/>
+      <c r="B86" s="5" t="inlineStr">
+        <is>
+          <t>N/A — no se elaboró un Diagrama de Secuencia dedicado para este requerimiento; el análisis se documenta como narrativa de caso de uso CU-016 (FD03, tabla de casos de uso — sin figura numerada, agregada en Sprint 13).</t>
+        </is>
+      </c>
+      <c r="C86" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D86" s="5" t="inlineStr">
+        <is>
+          <t>N/A — no se elaboró un Diagrama de Secuencia dedicado; el diseño se documenta como narrativa de caso de uso CU-007 (FD04, antes de §6 Vista Lógica — sin figura numerada, agregada en Sprint 13).</t>
+        </is>
+      </c>
+      <c r="E86" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F86" s="9" t="n"/>
+    </row>
+    <row r="87" ht="80" customHeight="1">
+      <c r="A87" s="9" t="n"/>
+      <c r="B87" s="5" t="inlineStr">
+        <is>
+          <t>N/A — no se elaboró un Diagrama de Actividades dedicado para este requerimiento; el análisis se documenta como narrativa de caso de uso CU-016 (FD03, tabla de casos de uso — sin figura numerada, agregada en Sprint 13).</t>
+        </is>
+      </c>
+      <c r="C87" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D87" s="5" t="inlineStr">
+        <is>
+          <t>N/A — no se elaboró un Diagrama de Actividades dedicado; el diseño se documenta como narrativa de caso de uso CU-007 (FD04, antes de §6 Vista Lógica — sin figura numerada, agregada en Sprint 13).</t>
+        </is>
+      </c>
+      <c r="E87" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F87" s="9" t="n"/>
+    </row>
+    <row r="88" ht="155" customHeight="1">
+      <c r="A88" s="10" t="n"/>
+      <c r="B88" s="5" t="inlineStr">
+        <is>
+          <t>N/A — el SRS (FD03) documenta el requerimiento a nivel de caso de uso; el modelo de datos persistente se define en la fase de diseño (FD04).</t>
+        </is>
+      </c>
+      <c r="C88" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D88" s="5" t="inlineStr">
+        <is>
+          <t>Diagrama de Entidad-Relación (lógico) — Base de Datos MongoDB.
+Entidad "WEARABLE_DATA" (colección wearabledata, índices { patientId, timestamp } y { timestamp }) — modelo ya existente desde antes de Sprint 13, tampoco representado en el Diagrama de Entidad-Relación documentado en DIAGRAMAS_MERMAID.md §4. La capa de validación (MedicalValidationRules.validate_vitals) es un motor de reglas sin estado propio, análogo a RF-005, que no persiste resultados adicionales.</t>
+        </is>
+      </c>
+      <c r="E88" s="6" t="inlineStr">
+        <is>
+          <t>→ Base para</t>
+        </is>
+      </c>
+      <c r="F88" s="10" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="27">

</xml_diff>